<commit_message>
Add environment doctor and template fields
</commit_message>
<xml_diff>
--- a/samples/DCP_v0.1/dataflow_collection_template_v0.1.xlsx
+++ b/samples/DCP_v0.1/dataflow_collection_template_v0.1.xlsx
@@ -207,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -355,6 +355,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1023,7 +1026,6 @@
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -1084,7 +1086,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
         <is>
@@ -1579,8 +1580,6 @@
       <c r="R2" s="1" t="n"/>
       <c r="S2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -2499,8 +2498,6 @@
       <c r="P2" s="1" t="n"/>
       <c r="Q2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -3427,8 +3424,6 @@
       <c r="Q2" s="1" t="n"/>
       <c r="R2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -4510,8 +4505,6 @@
       <c r="S2" s="1" t="n"/>
       <c r="T2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -5478,8 +5471,6 @@
       <c r="R2" s="1" t="n"/>
       <c r="S2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -6398,8 +6389,6 @@
       <c r="O2" s="1" t="n"/>
       <c r="P2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -7188,8 +7177,6 @@
       <c r="K2" s="1" t="n"/>
       <c r="L2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -10730,8 +10717,6 @@
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -11168,8 +11153,6 @@
       <c r="N2" s="1" t="n"/>
       <c r="O2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -11942,8 +11925,6 @@
       <c r="T2" s="1" t="n"/>
       <c r="U2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -13048,8 +13029,6 @@
       <c r="Y2" s="1" t="n"/>
       <c r="Z2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -14538,7 +14517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R39"/>
+  <dimension ref="A1:X39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14559,6 +14538,12 @@
     <col width="18" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="34" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -14584,6 +14569,12 @@
       <c r="P1" s="1" t="n"/>
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
@@ -14608,6 +14599,12 @@
       <c r="P2" s="1" t="n"/>
       <c r="Q2" s="1" t="n"/>
       <c r="R2" s="1" t="n"/>
+      <c r="S2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="n"/>
+      <c r="W2" s="1" t="n"/>
+      <c r="X2" s="1" t="n"/>
     </row>
     <row r="3"/>
     <row r="4"/>
@@ -14702,6 +14699,36 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="S5" s="64" t="inlineStr">
+        <is>
+          <t>Runtime_Type</t>
+        </is>
+      </c>
+      <c r="T5" s="64" t="inlineStr">
+        <is>
+          <t>Runtime_ID</t>
+        </is>
+      </c>
+      <c r="U5" s="64" t="inlineStr">
+        <is>
+          <t>Runtime_Name</t>
+        </is>
+      </c>
+      <c r="V5" s="64" t="inlineStr">
+        <is>
+          <t>Runtime_Namespace</t>
+        </is>
+      </c>
+      <c r="W5" s="64" t="inlineStr">
+        <is>
+          <t>Runtime_Cluster</t>
+        </is>
+      </c>
+      <c r="X5" s="64" t="inlineStr">
+        <is>
+          <t>Runtime_Region</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="43" t="inlineStr">
@@ -14790,6 +14817,12 @@
         </is>
       </c>
       <c r="R6" s="45" t="str"/>
+      <c r="S6" s="57" t="n"/>
+      <c r="T6" s="57" t="n"/>
+      <c r="U6" s="57" t="n"/>
+      <c r="V6" s="57" t="n"/>
+      <c r="W6" s="57" t="n"/>
+      <c r="X6" s="57" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="43" t="inlineStr">
@@ -14878,6 +14911,36 @@
         </is>
       </c>
       <c r="R7" s="45" t="str"/>
+      <c r="S7" s="57" t="inlineStr">
+        <is>
+          <t>Kubernetes</t>
+        </is>
+      </c>
+      <c r="T7" s="57" t="inlineStr">
+        <is>
+          <t>k8s-deploy-rpc</t>
+        </is>
+      </c>
+      <c r="U7" s="57" t="inlineStr">
+        <is>
+          <t>rpc-api-deployment</t>
+        </is>
+      </c>
+      <c r="V7" s="57" t="inlineStr">
+        <is>
+          <t>rpc</t>
+        </is>
+      </c>
+      <c r="W7" s="57" t="inlineStr">
+        <is>
+          <t>cluster-main</t>
+        </is>
+      </c>
+      <c r="X7" s="57" t="inlineStr">
+        <is>
+          <t>us-central1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="43" t="inlineStr">
@@ -14966,6 +15029,12 @@
         </is>
       </c>
       <c r="R8" s="45" t="str"/>
+      <c r="S8" s="57" t="n"/>
+      <c r="T8" s="57" t="n"/>
+      <c r="U8" s="57" t="n"/>
+      <c r="V8" s="57" t="n"/>
+      <c r="W8" s="57" t="n"/>
+      <c r="X8" s="57" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="43" t="inlineStr">
@@ -15054,6 +15123,12 @@
         </is>
       </c>
       <c r="R9" s="45" t="str"/>
+      <c r="S9" s="57" t="n"/>
+      <c r="T9" s="57" t="n"/>
+      <c r="U9" s="57" t="n"/>
+      <c r="V9" s="57" t="n"/>
+      <c r="W9" s="57" t="n"/>
+      <c r="X9" s="57" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="43" t="str"/>
@@ -15074,6 +15149,12 @@
       <c r="P10" s="44" t="str"/>
       <c r="Q10" s="62" t="str"/>
       <c r="R10" s="45" t="str"/>
+      <c r="S10" s="57" t="n"/>
+      <c r="T10" s="57" t="n"/>
+      <c r="U10" s="57" t="n"/>
+      <c r="V10" s="57" t="n"/>
+      <c r="W10" s="57" t="n"/>
+      <c r="X10" s="57" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="str"/>
@@ -15094,6 +15175,12 @@
       <c r="P11" s="44" t="str"/>
       <c r="Q11" s="62" t="str"/>
       <c r="R11" s="45" t="str"/>
+      <c r="S11" s="57" t="n"/>
+      <c r="T11" s="57" t="n"/>
+      <c r="U11" s="57" t="n"/>
+      <c r="V11" s="57" t="n"/>
+      <c r="W11" s="57" t="n"/>
+      <c r="X11" s="57" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="43" t="str"/>
@@ -15114,6 +15201,12 @@
       <c r="P12" s="44" t="str"/>
       <c r="Q12" s="62" t="str"/>
       <c r="R12" s="45" t="str"/>
+      <c r="S12" s="57" t="n"/>
+      <c r="T12" s="57" t="n"/>
+      <c r="U12" s="57" t="n"/>
+      <c r="V12" s="57" t="n"/>
+      <c r="W12" s="57" t="n"/>
+      <c r="X12" s="57" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="43" t="str"/>
@@ -15134,6 +15227,12 @@
       <c r="P13" s="44" t="str"/>
       <c r="Q13" s="62" t="str"/>
       <c r="R13" s="45" t="str"/>
+      <c r="S13" s="57" t="n"/>
+      <c r="T13" s="57" t="n"/>
+      <c r="U13" s="57" t="n"/>
+      <c r="V13" s="57" t="n"/>
+      <c r="W13" s="57" t="n"/>
+      <c r="X13" s="57" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="43" t="str"/>
@@ -15154,6 +15253,12 @@
       <c r="P14" s="44" t="str"/>
       <c r="Q14" s="62" t="str"/>
       <c r="R14" s="45" t="str"/>
+      <c r="S14" s="57" t="n"/>
+      <c r="T14" s="57" t="n"/>
+      <c r="U14" s="57" t="n"/>
+      <c r="V14" s="57" t="n"/>
+      <c r="W14" s="57" t="n"/>
+      <c r="X14" s="57" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="43" t="str"/>
@@ -15174,6 +15279,12 @@
       <c r="P15" s="44" t="str"/>
       <c r="Q15" s="62" t="str"/>
       <c r="R15" s="45" t="str"/>
+      <c r="S15" s="57" t="n"/>
+      <c r="T15" s="57" t="n"/>
+      <c r="U15" s="57" t="n"/>
+      <c r="V15" s="57" t="n"/>
+      <c r="W15" s="57" t="n"/>
+      <c r="X15" s="57" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="43" t="str"/>
@@ -15194,6 +15305,12 @@
       <c r="P16" s="44" t="str"/>
       <c r="Q16" s="62" t="str"/>
       <c r="R16" s="45" t="str"/>
+      <c r="S16" s="57" t="n"/>
+      <c r="T16" s="57" t="n"/>
+      <c r="U16" s="57" t="n"/>
+      <c r="V16" s="57" t="n"/>
+      <c r="W16" s="57" t="n"/>
+      <c r="X16" s="57" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="43" t="str"/>
@@ -15214,6 +15331,12 @@
       <c r="P17" s="44" t="str"/>
       <c r="Q17" s="62" t="str"/>
       <c r="R17" s="45" t="str"/>
+      <c r="S17" s="57" t="n"/>
+      <c r="T17" s="57" t="n"/>
+      <c r="U17" s="57" t="n"/>
+      <c r="V17" s="57" t="n"/>
+      <c r="W17" s="57" t="n"/>
+      <c r="X17" s="57" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="43" t="str"/>
@@ -15234,6 +15357,12 @@
       <c r="P18" s="44" t="str"/>
       <c r="Q18" s="62" t="str"/>
       <c r="R18" s="45" t="str"/>
+      <c r="S18" s="57" t="n"/>
+      <c r="T18" s="57" t="n"/>
+      <c r="U18" s="57" t="n"/>
+      <c r="V18" s="57" t="n"/>
+      <c r="W18" s="57" t="n"/>
+      <c r="X18" s="57" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="43" t="str"/>
@@ -15254,6 +15383,12 @@
       <c r="P19" s="44" t="str"/>
       <c r="Q19" s="62" t="str"/>
       <c r="R19" s="45" t="str"/>
+      <c r="S19" s="57" t="n"/>
+      <c r="T19" s="57" t="n"/>
+      <c r="U19" s="57" t="n"/>
+      <c r="V19" s="57" t="n"/>
+      <c r="W19" s="57" t="n"/>
+      <c r="X19" s="57" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="43" t="str"/>
@@ -15274,6 +15409,12 @@
       <c r="P20" s="44" t="str"/>
       <c r="Q20" s="62" t="str"/>
       <c r="R20" s="45" t="str"/>
+      <c r="S20" s="57" t="n"/>
+      <c r="T20" s="57" t="n"/>
+      <c r="U20" s="57" t="n"/>
+      <c r="V20" s="57" t="n"/>
+      <c r="W20" s="57" t="n"/>
+      <c r="X20" s="57" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="43" t="str"/>
@@ -15294,6 +15435,12 @@
       <c r="P21" s="44" t="str"/>
       <c r="Q21" s="62" t="str"/>
       <c r="R21" s="45" t="str"/>
+      <c r="S21" s="57" t="n"/>
+      <c r="T21" s="57" t="n"/>
+      <c r="U21" s="57" t="n"/>
+      <c r="V21" s="57" t="n"/>
+      <c r="W21" s="57" t="n"/>
+      <c r="X21" s="57" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="43" t="str"/>
@@ -15314,6 +15461,12 @@
       <c r="P22" s="44" t="str"/>
       <c r="Q22" s="62" t="str"/>
       <c r="R22" s="45" t="str"/>
+      <c r="S22" s="57" t="n"/>
+      <c r="T22" s="57" t="n"/>
+      <c r="U22" s="57" t="n"/>
+      <c r="V22" s="57" t="n"/>
+      <c r="W22" s="57" t="n"/>
+      <c r="X22" s="57" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="43" t="str"/>
@@ -15334,6 +15487,12 @@
       <c r="P23" s="44" t="str"/>
       <c r="Q23" s="62" t="str"/>
       <c r="R23" s="45" t="str"/>
+      <c r="S23" s="57" t="n"/>
+      <c r="T23" s="57" t="n"/>
+      <c r="U23" s="57" t="n"/>
+      <c r="V23" s="57" t="n"/>
+      <c r="W23" s="57" t="n"/>
+      <c r="X23" s="57" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="43" t="str"/>
@@ -15354,6 +15513,12 @@
       <c r="P24" s="44" t="str"/>
       <c r="Q24" s="62" t="str"/>
       <c r="R24" s="45" t="str"/>
+      <c r="S24" s="57" t="n"/>
+      <c r="T24" s="57" t="n"/>
+      <c r="U24" s="57" t="n"/>
+      <c r="V24" s="57" t="n"/>
+      <c r="W24" s="57" t="n"/>
+      <c r="X24" s="57" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="43" t="str"/>
@@ -15374,6 +15539,12 @@
       <c r="P25" s="44" t="str"/>
       <c r="Q25" s="62" t="str"/>
       <c r="R25" s="45" t="str"/>
+      <c r="S25" s="57" t="n"/>
+      <c r="T25" s="57" t="n"/>
+      <c r="U25" s="57" t="n"/>
+      <c r="V25" s="57" t="n"/>
+      <c r="W25" s="57" t="n"/>
+      <c r="X25" s="57" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="43" t="str"/>
@@ -15394,6 +15565,12 @@
       <c r="P26" s="44" t="str"/>
       <c r="Q26" s="62" t="str"/>
       <c r="R26" s="45" t="str"/>
+      <c r="S26" s="57" t="n"/>
+      <c r="T26" s="57" t="n"/>
+      <c r="U26" s="57" t="n"/>
+      <c r="V26" s="57" t="n"/>
+      <c r="W26" s="57" t="n"/>
+      <c r="X26" s="57" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="43" t="str"/>
@@ -15414,6 +15591,12 @@
       <c r="P27" s="44" t="str"/>
       <c r="Q27" s="62" t="str"/>
       <c r="R27" s="45" t="str"/>
+      <c r="S27" s="57" t="n"/>
+      <c r="T27" s="57" t="n"/>
+      <c r="U27" s="57" t="n"/>
+      <c r="V27" s="57" t="n"/>
+      <c r="W27" s="57" t="n"/>
+      <c r="X27" s="57" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="43" t="str"/>
@@ -15434,6 +15617,12 @@
       <c r="P28" s="44" t="str"/>
       <c r="Q28" s="62" t="str"/>
       <c r="R28" s="45" t="str"/>
+      <c r="S28" s="57" t="n"/>
+      <c r="T28" s="57" t="n"/>
+      <c r="U28" s="57" t="n"/>
+      <c r="V28" s="57" t="n"/>
+      <c r="W28" s="57" t="n"/>
+      <c r="X28" s="57" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="43" t="str"/>
@@ -15454,6 +15643,12 @@
       <c r="P29" s="44" t="str"/>
       <c r="Q29" s="62" t="str"/>
       <c r="R29" s="45" t="str"/>
+      <c r="S29" s="57" t="n"/>
+      <c r="T29" s="57" t="n"/>
+      <c r="U29" s="57" t="n"/>
+      <c r="V29" s="57" t="n"/>
+      <c r="W29" s="57" t="n"/>
+      <c r="X29" s="57" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="43" t="str"/>
@@ -15474,6 +15669,12 @@
       <c r="P30" s="44" t="str"/>
       <c r="Q30" s="62" t="str"/>
       <c r="R30" s="45" t="str"/>
+      <c r="S30" s="57" t="n"/>
+      <c r="T30" s="57" t="n"/>
+      <c r="U30" s="57" t="n"/>
+      <c r="V30" s="57" t="n"/>
+      <c r="W30" s="57" t="n"/>
+      <c r="X30" s="57" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="43" t="str"/>
@@ -15494,6 +15695,12 @@
       <c r="P31" s="44" t="str"/>
       <c r="Q31" s="62" t="str"/>
       <c r="R31" s="45" t="str"/>
+      <c r="S31" s="57" t="n"/>
+      <c r="T31" s="57" t="n"/>
+      <c r="U31" s="57" t="n"/>
+      <c r="V31" s="57" t="n"/>
+      <c r="W31" s="57" t="n"/>
+      <c r="X31" s="57" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="43" t="str"/>
@@ -15514,6 +15721,12 @@
       <c r="P32" s="44" t="str"/>
       <c r="Q32" s="62" t="str"/>
       <c r="R32" s="45" t="str"/>
+      <c r="S32" s="57" t="n"/>
+      <c r="T32" s="57" t="n"/>
+      <c r="U32" s="57" t="n"/>
+      <c r="V32" s="57" t="n"/>
+      <c r="W32" s="57" t="n"/>
+      <c r="X32" s="57" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="43" t="str"/>
@@ -15534,6 +15747,12 @@
       <c r="P33" s="44" t="str"/>
       <c r="Q33" s="62" t="str"/>
       <c r="R33" s="45" t="str"/>
+      <c r="S33" s="57" t="n"/>
+      <c r="T33" s="57" t="n"/>
+      <c r="U33" s="57" t="n"/>
+      <c r="V33" s="57" t="n"/>
+      <c r="W33" s="57" t="n"/>
+      <c r="X33" s="57" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="43" t="str"/>
@@ -15554,6 +15773,12 @@
       <c r="P34" s="44" t="str"/>
       <c r="Q34" s="62" t="str"/>
       <c r="R34" s="45" t="str"/>
+      <c r="S34" s="57" t="n"/>
+      <c r="T34" s="57" t="n"/>
+      <c r="U34" s="57" t="n"/>
+      <c r="V34" s="57" t="n"/>
+      <c r="W34" s="57" t="n"/>
+      <c r="X34" s="57" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="43" t="str"/>
@@ -15574,6 +15799,12 @@
       <c r="P35" s="44" t="str"/>
       <c r="Q35" s="62" t="str"/>
       <c r="R35" s="45" t="str"/>
+      <c r="S35" s="57" t="n"/>
+      <c r="T35" s="57" t="n"/>
+      <c r="U35" s="57" t="n"/>
+      <c r="V35" s="57" t="n"/>
+      <c r="W35" s="57" t="n"/>
+      <c r="X35" s="57" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="43" t="str"/>
@@ -15594,6 +15825,12 @@
       <c r="P36" s="44" t="str"/>
       <c r="Q36" s="62" t="str"/>
       <c r="R36" s="45" t="str"/>
+      <c r="S36" s="57" t="n"/>
+      <c r="T36" s="57" t="n"/>
+      <c r="U36" s="57" t="n"/>
+      <c r="V36" s="57" t="n"/>
+      <c r="W36" s="57" t="n"/>
+      <c r="X36" s="57" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="43" t="str"/>
@@ -15614,6 +15851,12 @@
       <c r="P37" s="44" t="str"/>
       <c r="Q37" s="62" t="str"/>
       <c r="R37" s="45" t="str"/>
+      <c r="S37" s="57" t="n"/>
+      <c r="T37" s="57" t="n"/>
+      <c r="U37" s="57" t="n"/>
+      <c r="V37" s="57" t="n"/>
+      <c r="W37" s="57" t="n"/>
+      <c r="X37" s="57" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="43" t="str"/>
@@ -15634,6 +15877,12 @@
       <c r="P38" s="44" t="str"/>
       <c r="Q38" s="62" t="str"/>
       <c r="R38" s="45" t="str"/>
+      <c r="S38" s="57" t="n"/>
+      <c r="T38" s="57" t="n"/>
+      <c r="U38" s="57" t="n"/>
+      <c r="V38" s="57" t="n"/>
+      <c r="W38" s="57" t="n"/>
+      <c r="X38" s="57" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="46" t="str"/>
@@ -15654,6 +15903,12 @@
       <c r="P39" s="47" t="str"/>
       <c r="Q39" s="63" t="str"/>
       <c r="R39" s="48" t="str"/>
+      <c r="S39" s="57" t="n"/>
+      <c r="T39" s="57" t="n"/>
+      <c r="U39" s="57" t="n"/>
+      <c r="V39" s="57" t="n"/>
+      <c r="W39" s="57" t="n"/>
+      <c r="X39" s="57" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -15690,7 +15945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T39"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15713,6 +15968,9 @@
     <col width="18" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -15740,6 +15998,9 @@
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
@@ -15766,6 +16027,9 @@
       <c r="R2" s="1" t="n"/>
       <c r="S2" s="1" t="n"/>
       <c r="T2" s="1" t="n"/>
+      <c r="U2" s="1" t="n"/>
+      <c r="V2" s="1" t="n"/>
+      <c r="W2" s="1" t="n"/>
     </row>
     <row r="3"/>
     <row r="4"/>
@@ -15870,6 +16134,21 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="U5" s="64" t="inlineStr">
+        <is>
+          <t>Target_Type</t>
+        </is>
+      </c>
+      <c r="V5" s="64" t="inlineStr">
+        <is>
+          <t>Target_ID</t>
+        </is>
+      </c>
+      <c r="W5" s="64" t="inlineStr">
+        <is>
+          <t>Interaction_Mode</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="43" t="inlineStr">
@@ -15958,6 +16237,21 @@
         </is>
       </c>
       <c r="T6" s="45" t="str"/>
+      <c r="U6" s="57" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="V6" s="57" t="inlineStr">
+        <is>
+          <t>svc-rpc-api</t>
+        </is>
+      </c>
+      <c r="W6" s="57" t="inlineStr">
+        <is>
+          <t>sync</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="43" t="inlineStr">
@@ -16042,6 +16336,21 @@
         </is>
       </c>
       <c r="T7" s="45" t="str"/>
+      <c r="U7" s="57" t="inlineStr">
+        <is>
+          <t>service</t>
+        </is>
+      </c>
+      <c r="V7" s="57" t="inlineStr">
+        <is>
+          <t>svc-sequencer</t>
+        </is>
+      </c>
+      <c r="W7" s="57" t="inlineStr">
+        <is>
+          <t>sync</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="43" t="inlineStr">
@@ -16126,6 +16435,21 @@
         </is>
       </c>
       <c r="T8" s="45" t="str"/>
+      <c r="U8" s="57" t="inlineStr">
+        <is>
+          <t>data_asset</t>
+        </is>
+      </c>
+      <c r="V8" s="57" t="inlineStr">
+        <is>
+          <t>data-cloudsql-state</t>
+        </is>
+      </c>
+      <c r="W8" s="57" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="43" t="inlineStr">
@@ -16216,6 +16540,21 @@
       <c r="T9" s="45" t="inlineStr">
         <is>
           <t>Endpoint requires confirmation</t>
+        </is>
+      </c>
+      <c r="U9" s="57" t="inlineStr">
+        <is>
+          <t>external_service</t>
+        </is>
+      </c>
+      <c r="V9" s="57" t="inlineStr">
+        <is>
+          <t>ext-eigenda</t>
+        </is>
+      </c>
+      <c r="W9" s="57" t="inlineStr">
+        <is>
+          <t>publish</t>
         </is>
       </c>
     </row>
@@ -16240,6 +16579,9 @@
       <c r="R10" s="44" t="str"/>
       <c r="S10" s="62" t="str"/>
       <c r="T10" s="45" t="str"/>
+      <c r="U10" s="57" t="n"/>
+      <c r="V10" s="57" t="n"/>
+      <c r="W10" s="57" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="43" t="str"/>
@@ -16262,6 +16604,9 @@
       <c r="R11" s="44" t="str"/>
       <c r="S11" s="62" t="str"/>
       <c r="T11" s="45" t="str"/>
+      <c r="U11" s="57" t="n"/>
+      <c r="V11" s="57" t="n"/>
+      <c r="W11" s="57" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="43" t="str"/>
@@ -16284,6 +16629,9 @@
       <c r="R12" s="44" t="str"/>
       <c r="S12" s="62" t="str"/>
       <c r="T12" s="45" t="str"/>
+      <c r="U12" s="57" t="n"/>
+      <c r="V12" s="57" t="n"/>
+      <c r="W12" s="57" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="43" t="str"/>
@@ -16306,6 +16654,9 @@
       <c r="R13" s="44" t="str"/>
       <c r="S13" s="62" t="str"/>
       <c r="T13" s="45" t="str"/>
+      <c r="U13" s="57" t="n"/>
+      <c r="V13" s="57" t="n"/>
+      <c r="W13" s="57" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="43" t="str"/>
@@ -16328,6 +16679,9 @@
       <c r="R14" s="44" t="str"/>
       <c r="S14" s="62" t="str"/>
       <c r="T14" s="45" t="str"/>
+      <c r="U14" s="57" t="n"/>
+      <c r="V14" s="57" t="n"/>
+      <c r="W14" s="57" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="43" t="str"/>
@@ -16350,6 +16704,9 @@
       <c r="R15" s="44" t="str"/>
       <c r="S15" s="62" t="str"/>
       <c r="T15" s="45" t="str"/>
+      <c r="U15" s="57" t="n"/>
+      <c r="V15" s="57" t="n"/>
+      <c r="W15" s="57" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="43" t="str"/>
@@ -16372,6 +16729,9 @@
       <c r="R16" s="44" t="str"/>
       <c r="S16" s="62" t="str"/>
       <c r="T16" s="45" t="str"/>
+      <c r="U16" s="57" t="n"/>
+      <c r="V16" s="57" t="n"/>
+      <c r="W16" s="57" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="43" t="str"/>
@@ -16394,6 +16754,9 @@
       <c r="R17" s="44" t="str"/>
       <c r="S17" s="62" t="str"/>
       <c r="T17" s="45" t="str"/>
+      <c r="U17" s="57" t="n"/>
+      <c r="V17" s="57" t="n"/>
+      <c r="W17" s="57" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="43" t="str"/>
@@ -16416,6 +16779,9 @@
       <c r="R18" s="44" t="str"/>
       <c r="S18" s="62" t="str"/>
       <c r="T18" s="45" t="str"/>
+      <c r="U18" s="57" t="n"/>
+      <c r="V18" s="57" t="n"/>
+      <c r="W18" s="57" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="43" t="str"/>
@@ -16438,6 +16804,9 @@
       <c r="R19" s="44" t="str"/>
       <c r="S19" s="62" t="str"/>
       <c r="T19" s="45" t="str"/>
+      <c r="U19" s="57" t="n"/>
+      <c r="V19" s="57" t="n"/>
+      <c r="W19" s="57" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="43" t="str"/>
@@ -16460,6 +16829,9 @@
       <c r="R20" s="44" t="str"/>
       <c r="S20" s="62" t="str"/>
       <c r="T20" s="45" t="str"/>
+      <c r="U20" s="57" t="n"/>
+      <c r="V20" s="57" t="n"/>
+      <c r="W20" s="57" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="43" t="str"/>
@@ -16482,6 +16854,9 @@
       <c r="R21" s="44" t="str"/>
       <c r="S21" s="62" t="str"/>
       <c r="T21" s="45" t="str"/>
+      <c r="U21" s="57" t="n"/>
+      <c r="V21" s="57" t="n"/>
+      <c r="W21" s="57" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="43" t="str"/>
@@ -16504,6 +16879,9 @@
       <c r="R22" s="44" t="str"/>
       <c r="S22" s="62" t="str"/>
       <c r="T22" s="45" t="str"/>
+      <c r="U22" s="57" t="n"/>
+      <c r="V22" s="57" t="n"/>
+      <c r="W22" s="57" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="43" t="str"/>
@@ -16526,6 +16904,9 @@
       <c r="R23" s="44" t="str"/>
       <c r="S23" s="62" t="str"/>
       <c r="T23" s="45" t="str"/>
+      <c r="U23" s="57" t="n"/>
+      <c r="V23" s="57" t="n"/>
+      <c r="W23" s="57" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="43" t="str"/>
@@ -16548,6 +16929,9 @@
       <c r="R24" s="44" t="str"/>
       <c r="S24" s="62" t="str"/>
       <c r="T24" s="45" t="str"/>
+      <c r="U24" s="57" t="n"/>
+      <c r="V24" s="57" t="n"/>
+      <c r="W24" s="57" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="43" t="str"/>
@@ -16570,6 +16954,9 @@
       <c r="R25" s="44" t="str"/>
       <c r="S25" s="62" t="str"/>
       <c r="T25" s="45" t="str"/>
+      <c r="U25" s="57" t="n"/>
+      <c r="V25" s="57" t="n"/>
+      <c r="W25" s="57" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="43" t="str"/>
@@ -16592,6 +16979,9 @@
       <c r="R26" s="44" t="str"/>
       <c r="S26" s="62" t="str"/>
       <c r="T26" s="45" t="str"/>
+      <c r="U26" s="57" t="n"/>
+      <c r="V26" s="57" t="n"/>
+      <c r="W26" s="57" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="43" t="str"/>
@@ -16614,6 +17004,9 @@
       <c r="R27" s="44" t="str"/>
       <c r="S27" s="62" t="str"/>
       <c r="T27" s="45" t="str"/>
+      <c r="U27" s="57" t="n"/>
+      <c r="V27" s="57" t="n"/>
+      <c r="W27" s="57" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="43" t="str"/>
@@ -16636,6 +17029,9 @@
       <c r="R28" s="44" t="str"/>
       <c r="S28" s="62" t="str"/>
       <c r="T28" s="45" t="str"/>
+      <c r="U28" s="57" t="n"/>
+      <c r="V28" s="57" t="n"/>
+      <c r="W28" s="57" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="43" t="str"/>
@@ -16658,6 +17054,9 @@
       <c r="R29" s="44" t="str"/>
       <c r="S29" s="62" t="str"/>
       <c r="T29" s="45" t="str"/>
+      <c r="U29" s="57" t="n"/>
+      <c r="V29" s="57" t="n"/>
+      <c r="W29" s="57" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="43" t="str"/>
@@ -16680,6 +17079,9 @@
       <c r="R30" s="44" t="str"/>
       <c r="S30" s="62" t="str"/>
       <c r="T30" s="45" t="str"/>
+      <c r="U30" s="57" t="n"/>
+      <c r="V30" s="57" t="n"/>
+      <c r="W30" s="57" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="43" t="str"/>
@@ -16702,6 +17104,9 @@
       <c r="R31" s="44" t="str"/>
       <c r="S31" s="62" t="str"/>
       <c r="T31" s="45" t="str"/>
+      <c r="U31" s="57" t="n"/>
+      <c r="V31" s="57" t="n"/>
+      <c r="W31" s="57" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="43" t="str"/>
@@ -16724,6 +17129,9 @@
       <c r="R32" s="44" t="str"/>
       <c r="S32" s="62" t="str"/>
       <c r="T32" s="45" t="str"/>
+      <c r="U32" s="57" t="n"/>
+      <c r="V32" s="57" t="n"/>
+      <c r="W32" s="57" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="43" t="str"/>
@@ -16746,6 +17154,9 @@
       <c r="R33" s="44" t="str"/>
       <c r="S33" s="62" t="str"/>
       <c r="T33" s="45" t="str"/>
+      <c r="U33" s="57" t="n"/>
+      <c r="V33" s="57" t="n"/>
+      <c r="W33" s="57" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="43" t="str"/>
@@ -16768,6 +17179,9 @@
       <c r="R34" s="44" t="str"/>
       <c r="S34" s="62" t="str"/>
       <c r="T34" s="45" t="str"/>
+      <c r="U34" s="57" t="n"/>
+      <c r="V34" s="57" t="n"/>
+      <c r="W34" s="57" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="43" t="str"/>
@@ -16790,6 +17204,9 @@
       <c r="R35" s="44" t="str"/>
       <c r="S35" s="62" t="str"/>
       <c r="T35" s="45" t="str"/>
+      <c r="U35" s="57" t="n"/>
+      <c r="V35" s="57" t="n"/>
+      <c r="W35" s="57" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="43" t="str"/>
@@ -16812,6 +17229,9 @@
       <c r="R36" s="44" t="str"/>
       <c r="S36" s="62" t="str"/>
       <c r="T36" s="45" t="str"/>
+      <c r="U36" s="57" t="n"/>
+      <c r="V36" s="57" t="n"/>
+      <c r="W36" s="57" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="43" t="str"/>
@@ -16834,6 +17254,9 @@
       <c r="R37" s="44" t="str"/>
       <c r="S37" s="62" t="str"/>
       <c r="T37" s="45" t="str"/>
+      <c r="U37" s="57" t="n"/>
+      <c r="V37" s="57" t="n"/>
+      <c r="W37" s="57" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="43" t="str"/>
@@ -16856,6 +17279,9 @@
       <c r="R38" s="44" t="str"/>
       <c r="S38" s="62" t="str"/>
       <c r="T38" s="45" t="str"/>
+      <c r="U38" s="57" t="n"/>
+      <c r="V38" s="57" t="n"/>
+      <c r="W38" s="57" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="46" t="str"/>
@@ -16878,6 +17304,9 @@
       <c r="R39" s="47" t="str"/>
       <c r="S39" s="63" t="str"/>
       <c r="T39" s="48" t="str"/>
+      <c r="U39" s="57" t="n"/>
+      <c r="V39" s="57" t="n"/>
+      <c r="W39" s="57" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -16994,8 +17423,6 @@
       <c r="T2" s="1" t="n"/>
       <c r="U2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>
@@ -18122,8 +18549,6 @@
       <c r="W2" s="1" t="n"/>
       <c r="X2" s="1" t="n"/>
     </row>
-    <row r="3"/>
-    <row r="4"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="40" t="inlineStr">
         <is>

</xml_diff>